<commit_message>
Update fig6 data and add immune protection analysis
Renamed 'CA' to 'CA (HPV)' in fig6_a_data.csv and corresponding R script for consistency. Updated fig6 figure files and Excel data. Enhanced 8_a_impact_factor.R to include immune protection as a factor in the analysis and updated data processing accordingly.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig6.xlsx
+++ b/Outcome/Publish/figure_data/fig6.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t xml:space="preserve">Shortname</t>
   </si>
@@ -64,6 +64,9 @@
     <t xml:space="preserve">Incubation_period</t>
   </si>
   <si>
+    <t xml:space="preserve">Immune_protection</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pneumonia</t>
   </si>
   <si>
@@ -76,6 +79,9 @@
     <t xml:space="preserve">Respiratory IDs</t>
   </si>
   <si>
+    <t xml:space="preserve">Short-term</t>
+  </si>
+  <si>
     <t xml:space="preserve">Influenza</t>
   </si>
   <si>
@@ -88,6 +94,9 @@
     <t xml:space="preserve">Chickenpox</t>
   </si>
   <si>
+    <t xml:space="preserve">Long-term</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mumps</t>
   </si>
   <si>
@@ -118,6 +127,9 @@
     <t xml:space="preserve">Melioidosis</t>
   </si>
   <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
     <t xml:space="preserve">S. suis</t>
   </si>
   <si>
@@ -151,7 +163,7 @@
     <t xml:space="preserve">HBV</t>
   </si>
   <si>
-    <t xml:space="preserve">CA</t>
+    <t xml:space="preserve">CA (HPV)</t>
   </si>
   <si>
     <t xml:space="preserve">Genital herpes</t>
@@ -221,6 +233,18 @@
   </si>
   <si>
     <t xml:space="preserve">VaccineOptional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immune_protectionLong-term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immune protection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immunity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immune_protectionShort-term</t>
   </si>
   <si>
     <t xml:space="preserve">Incubation Period</t>
@@ -257,9 +281,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -296,7 +318,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,10 +655,13 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>43922</v>
@@ -666,20 +691,23 @@
         <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O2"/>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>43891</v>
@@ -705,24 +733,27 @@
       </c>
       <c r="J3"/>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>1.55</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>43862</v>
@@ -748,24 +779,27 @@
       </c>
       <c r="J4"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L4" t="n">
         <v>11</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" t="n">
         <v>15</v>
       </c>
+      <c r="P4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>43831</v>
@@ -791,24 +825,27 @@
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L5" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O5" t="n">
         <v>17</v>
       </c>
+      <c r="P5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>43831</v>
@@ -834,24 +871,27 @@
       </c>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L6" t="n">
         <v>2.5</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O6" t="n">
         <v>3</v>
       </c>
+      <c r="P6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>43831</v>
@@ -875,24 +915,27 @@
       </c>
       <c r="J7"/>
       <c r="K7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L7" t="n">
         <v>6.5</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O7" t="n">
         <v>17</v>
       </c>
+      <c r="P7" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>43862</v>
@@ -918,24 +961,27 @@
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L8" t="n">
         <v>5</v>
       </c>
       <c r="M8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O8" t="n">
         <v>6</v>
       </c>
+      <c r="P8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>43983</v>
@@ -965,24 +1011,27 @@
         <v>6</v>
       </c>
       <c r="K9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O9" t="n">
         <v>11</v>
       </c>
+      <c r="P9" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>43891</v>
@@ -1012,24 +1061,27 @@
         <v>6</v>
       </c>
       <c r="K10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
         <v>8</v>
       </c>
+      <c r="P10" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>43922</v>
@@ -1059,24 +1111,27 @@
         <v>14</v>
       </c>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O11" t="n">
         <v>9</v>
       </c>
+      <c r="P11" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>43862</v>
@@ -1106,24 +1161,27 @@
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O12" t="n">
         <v>2</v>
       </c>
+      <c r="P12" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>43831</v>
@@ -1153,24 +1211,27 @@
         <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" t="n">
         <v>4</v>
       </c>
       <c r="M13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O13" t="n">
         <v>4</v>
       </c>
+      <c r="P13" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>44378</v>
@@ -1200,22 +1261,25 @@
         <v>8</v>
       </c>
       <c r="K14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L14"/>
       <c r="M14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O14" t="n">
         <v>2</v>
       </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>43891</v>
@@ -1241,24 +1305,27 @@
       </c>
       <c r="J15"/>
       <c r="K15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L15" t="n">
         <v>3.05</v>
       </c>
       <c r="M15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O15" t="n">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>43831</v>
@@ -1288,24 +1355,27 @@
         <v>25</v>
       </c>
       <c r="K16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L16" t="n">
         <v>3.7</v>
       </c>
       <c r="M16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N16" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O16" t="n">
         <v>10</v>
       </c>
+      <c r="P16" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>43831</v>
@@ -1331,24 +1401,27 @@
       </c>
       <c r="J17"/>
       <c r="K17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L17" t="n">
         <v>2.25</v>
       </c>
       <c r="M17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O17" t="n">
         <v>29</v>
       </c>
+      <c r="P17" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>43831</v>
@@ -1378,24 +1451,27 @@
         <v>28</v>
       </c>
       <c r="K18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L18" t="n">
         <v>2.75</v>
       </c>
       <c r="M18" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O18" t="n">
         <v>4</v>
       </c>
+      <c r="P18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>43952</v>
@@ -1419,24 +1495,27 @@
       </c>
       <c r="J19"/>
       <c r="K19" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L19" t="n">
         <v>1.6</v>
       </c>
       <c r="M19" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O19" t="n">
         <v>21</v>
       </c>
+      <c r="P19" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>43891</v>
@@ -1466,24 +1545,27 @@
         <v>15</v>
       </c>
       <c r="K20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L20" t="n">
         <v>6.5</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O20" t="n">
-        <v>45</v>
+        <v>90</v>
+      </c>
+      <c r="P20" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>43891</v>
@@ -1513,22 +1595,25 @@
         <v>14</v>
       </c>
       <c r="K21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L21"/>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N21" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O21" t="n">
         <v>90</v>
       </c>
+      <c r="P21" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>43862</v>
@@ -1558,24 +1643,27 @@
         <v>16</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L22" t="n">
         <v>2</v>
       </c>
       <c r="M22" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N22" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O22" t="n">
         <v>4</v>
       </c>
+      <c r="P22" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>43891</v>
@@ -1601,22 +1689,25 @@
       </c>
       <c r="J23"/>
       <c r="K23" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L23"/>
       <c r="M23" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O23" t="n">
         <v>6</v>
       </c>
+      <c r="P23" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>43831</v>
@@ -1646,19 +1737,22 @@
         <v>7</v>
       </c>
       <c r="K24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L24" t="n">
         <v>2.5</v>
       </c>
       <c r="M24" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N24" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
+      </c>
+      <c r="P24" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1718,10 +1812,13 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>43922</v>
@@ -1751,20 +1848,23 @@
         <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O2"/>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>43891</v>
@@ -1790,24 +1890,27 @@
       </c>
       <c r="J3"/>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>1.55</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>43862</v>
@@ -1833,24 +1936,27 @@
       </c>
       <c r="J4"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L4" t="n">
         <v>11</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" t="n">
         <v>15</v>
       </c>
+      <c r="P4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>43831</v>
@@ -1876,24 +1982,27 @@
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L5" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O5" t="n">
         <v>17</v>
       </c>
+      <c r="P5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>43831</v>
@@ -1919,24 +2028,27 @@
       </c>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L6" t="n">
         <v>2.5</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O6" t="n">
         <v>3</v>
       </c>
+      <c r="P6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>43831</v>
@@ -1960,24 +2072,27 @@
       </c>
       <c r="J7"/>
       <c r="K7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L7" t="n">
         <v>6.5</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O7" t="n">
         <v>17</v>
       </c>
+      <c r="P7" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>43862</v>
@@ -2003,24 +2118,27 @@
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L8" t="n">
         <v>5</v>
       </c>
       <c r="M8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O8" t="n">
         <v>6</v>
       </c>
+      <c r="P8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>43983</v>
@@ -2050,24 +2168,27 @@
         <v>6</v>
       </c>
       <c r="K9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O9" t="n">
         <v>11</v>
       </c>
+      <c r="P9" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>43891</v>
@@ -2097,24 +2218,27 @@
         <v>6</v>
       </c>
       <c r="K10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
         <v>8</v>
       </c>
+      <c r="P10" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>43922</v>
@@ -2144,24 +2268,27 @@
         <v>14</v>
       </c>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O11" t="n">
         <v>9</v>
       </c>
+      <c r="P11" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>43862</v>
@@ -2191,24 +2318,27 @@
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O12" t="n">
         <v>2</v>
       </c>
+      <c r="P12" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>43831</v>
@@ -2238,24 +2368,27 @@
         <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" t="n">
         <v>4</v>
       </c>
       <c r="M13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O13" t="n">
         <v>4</v>
       </c>
+      <c r="P13" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>44378</v>
@@ -2285,22 +2418,25 @@
         <v>8</v>
       </c>
       <c r="K14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L14"/>
       <c r="M14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O14" t="n">
         <v>2</v>
       </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>43891</v>
@@ -2326,24 +2462,27 @@
       </c>
       <c r="J15"/>
       <c r="K15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L15" t="n">
         <v>3.05</v>
       </c>
       <c r="M15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O15" t="n">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>43831</v>
@@ -2373,24 +2512,27 @@
         <v>25</v>
       </c>
       <c r="K16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L16" t="n">
         <v>3.7</v>
       </c>
       <c r="M16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N16" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O16" t="n">
         <v>10</v>
       </c>
+      <c r="P16" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>43831</v>
@@ -2416,24 +2558,27 @@
       </c>
       <c r="J17"/>
       <c r="K17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L17" t="n">
         <v>2.25</v>
       </c>
       <c r="M17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O17" t="n">
         <v>29</v>
       </c>
+      <c r="P17" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>43831</v>
@@ -2463,24 +2608,27 @@
         <v>28</v>
       </c>
       <c r="K18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L18" t="n">
         <v>2.75</v>
       </c>
       <c r="M18" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O18" t="n">
         <v>4</v>
       </c>
+      <c r="P18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>43952</v>
@@ -2504,24 +2652,27 @@
       </c>
       <c r="J19"/>
       <c r="K19" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L19" t="n">
         <v>1.6</v>
       </c>
       <c r="M19" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O19" t="n">
         <v>21</v>
       </c>
+      <c r="P19" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>43891</v>
@@ -2551,24 +2702,27 @@
         <v>15</v>
       </c>
       <c r="K20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L20" t="n">
         <v>6.5</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O20" t="n">
-        <v>45</v>
+        <v>90</v>
+      </c>
+      <c r="P20" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>43891</v>
@@ -2598,22 +2752,25 @@
         <v>14</v>
       </c>
       <c r="K21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L21"/>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N21" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O21" t="n">
         <v>90</v>
       </c>
+      <c r="P21" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>43862</v>
@@ -2643,24 +2800,27 @@
         <v>16</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L22" t="n">
         <v>2</v>
       </c>
       <c r="M22" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N22" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O22" t="n">
         <v>4</v>
       </c>
+      <c r="P22" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>43891</v>
@@ -2686,22 +2846,25 @@
       </c>
       <c r="J23"/>
       <c r="K23" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L23"/>
       <c r="M23" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O23" t="n">
         <v>6</v>
       </c>
+      <c r="P23" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>43831</v>
@@ -2731,19 +2894,22 @@
         <v>7</v>
       </c>
       <c r="K24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L24" t="n">
         <v>2.5</v>
       </c>
       <c r="M24" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N24" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
+      </c>
+      <c r="P24" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2803,10 +2969,13 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>43922</v>
@@ -2836,20 +3005,23 @@
         <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O2"/>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>43891</v>
@@ -2875,24 +3047,27 @@
       </c>
       <c r="J3"/>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>1.55</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>43862</v>
@@ -2918,24 +3093,27 @@
       </c>
       <c r="J4"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L4" t="n">
         <v>11</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" t="n">
         <v>15</v>
       </c>
+      <c r="P4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>43831</v>
@@ -2961,24 +3139,27 @@
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L5" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O5" t="n">
         <v>17</v>
       </c>
+      <c r="P5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>43831</v>
@@ -3004,24 +3185,27 @@
       </c>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L6" t="n">
         <v>2.5</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O6" t="n">
         <v>3</v>
       </c>
+      <c r="P6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>43831</v>
@@ -3045,24 +3229,27 @@
       </c>
       <c r="J7"/>
       <c r="K7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L7" t="n">
         <v>6.5</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O7" t="n">
         <v>17</v>
       </c>
+      <c r="P7" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>43862</v>
@@ -3088,24 +3275,27 @@
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L8" t="n">
         <v>5</v>
       </c>
       <c r="M8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O8" t="n">
         <v>6</v>
       </c>
+      <c r="P8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>43983</v>
@@ -3135,24 +3325,27 @@
         <v>6</v>
       </c>
       <c r="K9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O9" t="n">
         <v>11</v>
       </c>
+      <c r="P9" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>43891</v>
@@ -3182,24 +3375,27 @@
         <v>6</v>
       </c>
       <c r="K10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
         <v>8</v>
       </c>
+      <c r="P10" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>43922</v>
@@ -3229,24 +3425,27 @@
         <v>14</v>
       </c>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O11" t="n">
         <v>9</v>
       </c>
+      <c r="P11" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>43862</v>
@@ -3276,24 +3475,27 @@
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O12" t="n">
         <v>2</v>
       </c>
+      <c r="P12" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>43831</v>
@@ -3323,24 +3525,27 @@
         <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" t="n">
         <v>4</v>
       </c>
       <c r="M13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O13" t="n">
         <v>4</v>
       </c>
+      <c r="P13" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>44378</v>
@@ -3370,22 +3575,25 @@
         <v>8</v>
       </c>
       <c r="K14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L14"/>
       <c r="M14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O14" t="n">
         <v>2</v>
       </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>43891</v>
@@ -3411,24 +3619,27 @@
       </c>
       <c r="J15"/>
       <c r="K15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L15" t="n">
         <v>3.05</v>
       </c>
       <c r="M15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O15" t="n">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>43831</v>
@@ -3458,24 +3669,27 @@
         <v>25</v>
       </c>
       <c r="K16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L16" t="n">
         <v>3.7</v>
       </c>
       <c r="M16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N16" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O16" t="n">
         <v>10</v>
       </c>
+      <c r="P16" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>43831</v>
@@ -3501,24 +3715,27 @@
       </c>
       <c r="J17"/>
       <c r="K17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L17" t="n">
         <v>2.25</v>
       </c>
       <c r="M17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O17" t="n">
         <v>29</v>
       </c>
+      <c r="P17" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>43831</v>
@@ -3548,24 +3765,27 @@
         <v>28</v>
       </c>
       <c r="K18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L18" t="n">
         <v>2.75</v>
       </c>
       <c r="M18" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O18" t="n">
         <v>4</v>
       </c>
+      <c r="P18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>43952</v>
@@ -3589,24 +3809,27 @@
       </c>
       <c r="J19"/>
       <c r="K19" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L19" t="n">
         <v>1.6</v>
       </c>
       <c r="M19" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O19" t="n">
         <v>21</v>
       </c>
+      <c r="P19" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>43891</v>
@@ -3636,24 +3859,27 @@
         <v>15</v>
       </c>
       <c r="K20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L20" t="n">
         <v>6.5</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O20" t="n">
-        <v>45</v>
+        <v>90</v>
+      </c>
+      <c r="P20" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>43891</v>
@@ -3683,22 +3909,25 @@
         <v>14</v>
       </c>
       <c r="K21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L21"/>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N21" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O21" t="n">
         <v>90</v>
       </c>
+      <c r="P21" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>43862</v>
@@ -3728,24 +3957,27 @@
         <v>16</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L22" t="n">
         <v>2</v>
       </c>
       <c r="M22" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N22" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O22" t="n">
         <v>4</v>
       </c>
+      <c r="P22" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>43891</v>
@@ -3771,22 +4003,25 @@
       </c>
       <c r="J23"/>
       <c r="K23" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L23"/>
       <c r="M23" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O23" t="n">
         <v>6</v>
       </c>
+      <c r="P23" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>43831</v>
@@ -3816,19 +4051,22 @@
         <v>7</v>
       </c>
       <c r="K24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L24" t="n">
         <v>2.5</v>
       </c>
       <c r="M24" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N24" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
+      </c>
+      <c r="P24" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3844,42 +4082,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B2" t="n">
         <v>12.3633051962839</v>
@@ -3900,13 +4138,13 @@
         <v>53.911651510797</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="K2" t="n">
         <v>1</v>
@@ -3914,7 +4152,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B3" t="n">
         <v>1.90130131081289</v>
@@ -3935,13 +4173,13 @@
         <v>6.45937211499753</v>
       </c>
       <c r="H3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="K3" t="n">
         <v>2</v>
@@ -3949,7 +4187,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B4" t="n">
         <v>5.2254081310057</v>
@@ -3970,13 +4208,13 @@
         <v>20.1472584989017</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K4" t="n">
         <v>3</v>
@@ -3994,10 +4232,10 @@
       <c r="G5"/>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K5" t="n">
         <v>4</v>
@@ -4005,7 +4243,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B6" t="n">
         <v>0.477647176270998</v>
@@ -4026,13 +4264,13 @@
         <v>1.51431830466338</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
@@ -4040,7 +4278,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" t="n">
         <v>0.933345447955987</v>
@@ -4061,13 +4299,13 @@
         <v>2.5634538205906</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K7" t="n">
         <v>6</v>
@@ -4085,10 +4323,10 @@
       <c r="G8"/>
       <c r="H8"/>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K8" t="n">
         <v>7</v>
@@ -4096,34 +4334,34 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>72</v>
       </c>
       <c r="B9" t="n">
-        <v>1.00004845265542</v>
+        <v>0.509465307621857</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0100114537830617</v>
+        <v>0.611449881600934</v>
       </c>
       <c r="D9" t="n">
-        <v>0.00483960498434717</v>
+        <v>-1.10294161460739</v>
       </c>
       <c r="E9" t="n">
-        <v>0.996138568976206</v>
+        <v>0.270052520815003</v>
       </c>
       <c r="F9" t="n">
-        <v>0.98061668250031</v>
+        <v>0.153690680296362</v>
       </c>
       <c r="G9" t="n">
-        <v>1.01986528019136</v>
+        <v>1.68881352577614</v>
       </c>
       <c r="H9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="K9" t="n">
         <v>8</v>
@@ -4131,37 +4369,128 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="B10" t="n">
-        <v>0.957494439139157</v>
+        <v>1.54403144795736</v>
       </c>
       <c r="C10" t="n">
-        <v>0.100764731184389</v>
+        <v>0.522018973706555</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.431057227278091</v>
+        <v>0.832147567661747</v>
       </c>
       <c r="E10" t="n">
-        <v>0.666426760237564</v>
+        <v>0.405325655044071</v>
       </c>
       <c r="F10" t="n">
-        <v>0.785896158094</v>
+        <v>0.555025306782904</v>
       </c>
       <c r="G10" t="n">
-        <v>1.16656073647933</v>
+        <v>4.29535929829916</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="J10" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="K10" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11"/>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1.00025207331743</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.00877061758567438</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.0287370358845847</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.977074318191719</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.983204589285983</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.01759513846696</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I12" t="s">
+        <v>77</v>
+      </c>
+      <c r="J12" t="s">
+        <v>77</v>
+      </c>
+      <c r="K12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.961805508716482</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0837912785878094</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.464762243804498</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.642101728597364</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.816138742499317</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.13347129406511</v>
+      </c>
+      <c r="H13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" t="s">
+        <v>78</v>
+      </c>
+      <c r="J13" t="s">
+        <v>79</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -4221,10 +4550,13 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>43922</v>
@@ -4254,20 +4586,23 @@
         <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O2"/>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>43891</v>
@@ -4293,24 +4628,27 @@
       </c>
       <c r="J3"/>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>1.55</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>43831</v>
@@ -4336,24 +4674,27 @@
       </c>
       <c r="J4"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L4" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="M4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" t="n">
         <v>17</v>
       </c>
+      <c r="P4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>43831</v>
@@ -4379,24 +4720,27 @@
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L5" t="n">
         <v>2.5</v>
       </c>
       <c r="M5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O5" t="n">
         <v>3</v>
       </c>
+      <c r="P5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>43862</v>
@@ -4422,24 +4766,27 @@
       </c>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L6" t="n">
         <v>5</v>
       </c>
       <c r="M6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O6" t="n">
         <v>6</v>
       </c>
+      <c r="P6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>43983</v>
@@ -4469,24 +4816,27 @@
         <v>6</v>
       </c>
       <c r="K7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O7" t="n">
         <v>11</v>
       </c>
+      <c r="P7" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>43891</v>
@@ -4516,24 +4866,27 @@
         <v>6</v>
       </c>
       <c r="K8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O8" t="n">
         <v>8</v>
       </c>
+      <c r="P8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>43922</v>
@@ -4563,24 +4916,27 @@
         <v>14</v>
       </c>
       <c r="K9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O9" t="n">
         <v>9</v>
       </c>
+      <c r="P9" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>43862</v>
@@ -4610,24 +4966,27 @@
         <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
         <v>2</v>
       </c>
+      <c r="P10" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>43831</v>
@@ -4657,24 +5016,27 @@
         <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L11" t="n">
         <v>4</v>
       </c>
       <c r="M11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O11" t="n">
         <v>4</v>
       </c>
+      <c r="P11" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>44378</v>
@@ -4704,22 +5066,25 @@
         <v>8</v>
       </c>
       <c r="K12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L12"/>
       <c r="M12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O12" t="n">
         <v>2</v>
       </c>
+      <c r="P12" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>43891</v>
@@ -4745,24 +5110,27 @@
       </c>
       <c r="J13"/>
       <c r="K13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L13" t="n">
         <v>3.05</v>
       </c>
       <c r="M13" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O13" t="n">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="P13" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>43831</v>
@@ -4792,24 +5160,27 @@
         <v>25</v>
       </c>
       <c r="K14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L14" t="n">
         <v>3.7</v>
       </c>
       <c r="M14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O14" t="n">
         <v>10</v>
       </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>43831</v>
@@ -4835,24 +5206,27 @@
       </c>
       <c r="J15"/>
       <c r="K15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L15" t="n">
         <v>2.25</v>
       </c>
       <c r="M15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O15" t="n">
         <v>29</v>
       </c>
+      <c r="P15" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>43831</v>
@@ -4882,24 +5256,27 @@
         <v>28</v>
       </c>
       <c r="K16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L16" t="n">
         <v>2.75</v>
       </c>
       <c r="M16" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N16" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O16" t="n">
         <v>4</v>
       </c>
+      <c r="P16" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>43891</v>
@@ -4929,24 +5306,27 @@
         <v>15</v>
       </c>
       <c r="K17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L17" t="n">
         <v>6.5</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N17" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O17" t="n">
-        <v>45</v>
+        <v>90</v>
+      </c>
+      <c r="P17" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>43891</v>
@@ -4976,22 +5356,25 @@
         <v>14</v>
       </c>
       <c r="K18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L18"/>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O18" t="n">
         <v>90</v>
       </c>
+      <c r="P18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>43862</v>
@@ -5021,24 +5404,27 @@
         <v>16</v>
       </c>
       <c r="K19" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L19" t="n">
         <v>2</v>
       </c>
       <c r="M19" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O19" t="n">
         <v>4</v>
       </c>
+      <c r="P19" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>43891</v>
@@ -5064,22 +5450,25 @@
       </c>
       <c r="J20"/>
       <c r="K20" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L20"/>
       <c r="M20" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
       </c>
+      <c r="P20" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>43831</v>
@@ -5109,19 +5498,22 @@
         <v>7</v>
       </c>
       <c r="K21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L21" t="n">
         <v>2.5</v>
       </c>
       <c r="M21" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N21" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O21" t="n">
         <v>100</v>
+      </c>
+      <c r="P21" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -5146,13 +5538,13 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="E1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="F1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G1" t="s">
         <v>13</v>
@@ -5160,7 +5552,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" t="n">
         <v>-0.279365719412144</v>
@@ -5175,15 +5567,15 @@
         <v>0.106994709622438</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" t="n">
         <v>-0.825178955136324</v>
@@ -5198,15 +5590,15 @@
         <v>0.261305452583169</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" t="n">
         <v>-0.531646569095555</v>
@@ -5221,15 +5613,15 @@
         <v>0.185158562424776</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" t="n">
         <v>-0.532969487397903</v>
@@ -5244,15 +5636,15 @@
         <v>0.185533510636111</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" t="n">
         <v>-0.752979061768441</v>
@@ -5267,15 +5659,15 @@
         <v>0.243776728750535</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" t="n">
         <v>-0.820183931677406</v>
@@ -5290,15 +5682,15 @@
         <v>0.260115276158921</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" t="n">
         <v>-0.520828806653862</v>
@@ -5313,15 +5705,15 @@
         <v>0.182080330088535</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" t="n">
         <v>-0.162131326836121</v>
@@ -5336,15 +5728,15 @@
         <v>0.0652552083447888</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" t="n">
         <v>-0.263097876618642</v>
@@ -5359,15 +5751,15 @@
         <v>0.101437005051301</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" t="n">
         <v>-0.157386998715913</v>
@@ -5382,15 +5774,15 @@
         <v>0.0634785994914555</v>
       </c>
       <c r="F11" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B12" t="n">
         <v>-0.182195878553904</v>
@@ -5405,15 +5797,15 @@
         <v>0.0726894409505976</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B13" t="n">
         <v>-0.434848324854664</v>
@@ -5428,15 +5820,15 @@
         <v>0.156805995035081</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" t="n">
         <v>-0.0840752991672098</v>
@@ -5451,15 +5843,15 @@
         <v>0.0350594490631195</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" t="n">
         <v>-0.193486895277608</v>
@@ -5474,15 +5866,15 @@
         <v>0.0768176547295621</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B16" t="n">
         <v>-0.483975972467514</v>
@@ -5497,15 +5889,15 @@
         <v>0.17142686919823</v>
       </c>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G16" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" t="n">
         <v>-0.359868960587593</v>
@@ -5520,15 +5912,15 @@
         <v>0.133497060991106</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B18" t="n">
         <v>-0.343081309845054</v>
@@ -5543,15 +5935,15 @@
         <v>0.12810230555636</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" t="n">
         <v>-0.253217630155129</v>
@@ -5566,15 +5958,15 @@
         <v>0.0980264958691239</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B20" t="n">
         <v>-0.208147748441247</v>
@@ -5589,15 +5981,15 @@
         <v>0.0821200488621207</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" t="n">
         <v>-0.232350403525653</v>
@@ -5612,15 +6004,15 @@
         <v>0.0907342116275728</v>
       </c>
       <c r="F21" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G21" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" t="n">
         <v>-0.244260507517835</v>
@@ -5635,15 +6027,15 @@
         <v>0.0949113169569454</v>
       </c>
       <c r="F22" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G22" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B23" t="n">
         <v>-0.2446250364635</v>
@@ -5658,10 +6050,10 @@
         <v>0.0950385328597509</v>
       </c>
       <c r="F23" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>